<commit_message>
feat: update sample data with dirty records to exercise the cleaning pipeline
</commit_message>
<xml_diff>
--- a/data/raw/sales_february.xlsx
+++ b/data/raw/sales_february.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:F6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -496,7 +496,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>North</t>
+          <t>north</t>
         </is>
       </c>
     </row>
@@ -523,6 +523,54 @@
       <c r="F4" t="inlineStr">
         <is>
           <t>South</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2024-02-10</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr"/>
+      <c r="C5" t="n">
+        <v>5</v>
+      </c>
+      <c r="D5" t="n">
+        <v>25</v>
+      </c>
+      <c r="E5" t="inlineStr"/>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>East</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2024-02-20</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>widget a</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>25</v>
+      </c>
+      <c r="E6" t="n">
+        <v>100</v>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  NORTH  </t>
         </is>
       </c>
     </row>

</xml_diff>